<commit_message>
Update BOM and CPL files for RheoBoard V1
- Revised `BOM_RheoboardV1_JLCSMT.xlsx` and `CPL_JLCSMT.xlsx` to include updated component data, ensuring accuracy in sourcing.
- Modified `CPL.csv` to adjust the footprint coordinates for component F1, enhancing the precision of the design files.

These updates improve project documentation and maintain the relevance of the BOM and CPL for users.
</commit_message>
<xml_diff>
--- a/RheoBoard_PCB/RheoBoard_v1/CPL/CPL_JLCSMT.xlsx
+++ b/RheoBoard_PCB/RheoBoard_v1/CPL/CPL_JLCSMT.xlsx
@@ -1872,12 +1872,12 @@
       </c>
       <c r="B58" s="2" t="inlineStr">
         <is>
-          <t>125.3000mm</t>
+          <t>127.2000mm</t>
         </is>
       </c>
       <c r="C58" s="2" t="inlineStr">
         <is>
-          <t>-53.3700mm</t>
+          <t>-58.7300mm</t>
         </is>
       </c>
       <c r="D58" s="2" t="inlineStr">

</xml_diff>